<commit_message>
Layout changes and bug fixes
</commit_message>
<xml_diff>
--- a/public/LinearModule.xlsx
+++ b/public/LinearModule.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ru0nntr\Desktop\Прочее\Linear Motion Calculator\project_v0.96\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ru0nntr\Desktop\Прочее\Linear Motion Calculator\project_v0.97\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -1498,7 +1498,7 @@
         <v>5</v>
       </c>
       <c r="C17">
-        <v>0.4</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="D17">
         <v>1.5E-6</v>
@@ -1555,7 +1555,7 @@
         <v>10</v>
       </c>
       <c r="C18">
-        <v>0.4</v>
+        <v>0.08</v>
       </c>
       <c r="D18">
         <v>1.5E-6</v>
@@ -1612,7 +1612,7 @@
         <v>20</v>
       </c>
       <c r="C19">
-        <v>0.4</v>
+        <v>0.09</v>
       </c>
       <c r="D19">
         <v>1.5E-6</v>
@@ -1669,7 +1669,7 @@
         <v>5</v>
       </c>
       <c r="C20">
-        <v>0.75</v>
+        <v>0.1</v>
       </c>
       <c r="D20">
         <v>9.9999999999999991E-6</v>
@@ -1725,7 +1725,7 @@
         <v>10</v>
       </c>
       <c r="C21">
-        <v>0.75</v>
+        <v>0.12</v>
       </c>
       <c r="D21">
         <v>9.9999999999999991E-6</v>
@@ -1781,7 +1781,7 @@
         <v>20</v>
       </c>
       <c r="C22">
-        <v>0.75</v>
+        <v>0.15</v>
       </c>
       <c r="D22">
         <v>9.9999999999999991E-6</v>
@@ -1837,7 +1837,7 @@
         <v>32</v>
       </c>
       <c r="C23">
-        <v>0.75</v>
+        <v>0.17</v>
       </c>
       <c r="D23">
         <v>9.9999999999999991E-6</v>
@@ -1893,7 +1893,7 @@
         <v>5</v>
       </c>
       <c r="C24">
-        <v>1.3</v>
+        <v>0.12</v>
       </c>
       <c r="D24">
         <v>6.4459999999999989E-5</v>
@@ -1949,7 +1949,7 @@
         <v>10</v>
       </c>
       <c r="C25">
-        <v>1.3</v>
+        <v>0.15</v>
       </c>
       <c r="D25">
         <v>6.4459999999999989E-5</v>
@@ -2005,7 +2005,7 @@
         <v>20</v>
       </c>
       <c r="C26">
-        <v>1.3</v>
+        <v>0.17</v>
       </c>
       <c r="D26">
         <v>6.4459999999999989E-5</v>
@@ -2061,7 +2061,7 @@
         <v>32</v>
       </c>
       <c r="C27">
-        <v>1.3</v>
+        <v>0.19</v>
       </c>
       <c r="D27">
         <v>6.4459999999999989E-5</v>

</xml_diff>